<commit_message>
Agregar columna 'Materias primas exportadas' al Excel
</commit_message>
<xml_diff>
--- a/BD_banderas.xlsx
+++ b/BD_banderas.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,7 @@
     <col width="24" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,6 +547,11 @@
           <t>Significado escudo</t>
         </is>
       </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Materias primas exportadas</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="80" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -603,6 +609,11 @@
           <t>Dos manos entrelazadas sostienen una pica con el gorro frigio, símbolo de libertad. Arriba brilla el Sol de Mayo. El laurel alrededor representa la victoria.</t>
         </is>
       </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Soja, maíz, carne vacuna, trigo</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="80" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -660,6 +671,11 @@
           <t>Muestra el cerro Potosí (riqueza mineral), una alpaca (fauna), el árbol del pan (agricultura) y un sol naciente sobre montañas. Rodeado por banderas y cañones.</t>
         </is>
       </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Gas natural, zinc, estaño, plata</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -717,6 +733,11 @@
           <t>Una estrella de cinco puntas con la Cruz del Sur, rodeada de café y tabaco (productos clave), sobre una espada que representa la defensa de la República.</t>
         </is>
       </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Soja, mineral de hierro, petróleo, café</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -774,6 +795,11 @@
           <t>Combina los símbolos de Inglaterra (leones), Escocia (león rampante), Irlanda (arpa) y Francia (flores de lis), sobre hojas de arce rojas.</t>
         </is>
       </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, oro, madera, trigo</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -831,6 +857,11 @@
           <t>Sostenido por un cóndor (aire) y un huemul (tierra). La estrella sobre fondo azul y rojo representa la soberanía. El lema: 'Por la razón o la fuerza'.</t>
         </is>
       </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Cobre, litio, frutas, salmón</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -888,6 +919,11 @@
           <t>Muestra una granada dorada (origen del nombre Nueva Granada), un cóndor coronado con laureles y los dos mares con barcos, símbolo del comercio.</t>
         </is>
       </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, café, carbón, flores</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -945,6 +981,11 @@
           <t>Muestra tres volcanes entre dos océanos con barcos, representando el istmo. Las siete estrellas son las siete provincias del país.</t>
         </is>
       </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Dispositivos médicos, banano, piña, café</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
@@ -1002,6 +1043,11 @@
           <t>Contiene una llave dorada (Cuba, 'llave del Golfo'), un sol naciente, una palma real (el pueblo) y montañas. Rodeado por una rama de roble y otra de laurel.</t>
         </is>
       </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Níquel, tabaco, azúcar, ron</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
@@ -1059,6 +1105,11 @@
           <t>El volcán Chimborazo y el río Guayas con un barco (comercio). Arriba, un sol dorado entre los signos del zodiaco (meses de gestas patrióticas).</t>
         </is>
       </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, banano, camarón, cacao</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
@@ -1116,6 +1167,11 @@
           <t>Un águila calva (símbolo nacional) sostiene 13 flechas (guerra) y una rama de olivo (paz). En su pico lleva el lema 'E Pluribus Unum' ('De muchos, uno').</t>
         </is>
       </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, aviones, maíz, soja</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
@@ -1173,6 +1229,11 @@
           <t>Destacan un quetzal (ave nacional y símbolo de libertad), un pergamino con la fecha de la independencia y dos fusiles cruzados sobre ramas de laurel.</t>
         </is>
       </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Café, azúcar, banano, cardamomo</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -1230,6 +1291,11 @@
           <t>Un águila real parada sobre un nopal devorando una serpiente, recordando la leyenda de la fundación de Tenochtitlán por los mexicas.</t>
         </is>
       </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, petróleo, electrónica, aguacate</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
@@ -1287,6 +1353,11 @@
           <t>Muestra un rifle y una espada colgados (fin de las guerras civiles), una pala y un azadón (el trabajo), y un istmo entre dos océanos con un sol y la luna.</t>
         </is>
       </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Cobre, banano, azúcar, café</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
@@ -1344,6 +1415,11 @@
           <t>Tres campos: una vicuña (fauna andina), un árbol de la quina (flora) y una cornucopia con monedas de oro (las riquezas minerales del Perú).</t>
         </is>
       </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Cobre, oro, zinc, harina de pescado</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="80" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
@@ -1401,6 +1477,11 @@
           <t>Una estrella amarilla rodeada por una palma y un olivo, bajo la leyenda 'República del Paraguay'. Simboliza paz, gloria y soberanía.</t>
         </is>
       </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Soja, carne vacuna, maíz, energía eléctrica</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="80" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
@@ -1458,6 +1539,11 @@
           <t>Dividido en cuatro cuarteles: una balanza (igualdad y justicia), el Cerro de Montevideo (fuerza), un caballo suelto (libertad) y un buey (abundancia).</t>
         </is>
       </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Carne vacuna, soja, celulosa, lácteos</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
@@ -1515,6 +1601,11 @@
           <t>Un águila negra ('Bundesadler') sobre fondo dorado. Es uno de los símbolos heráldicos más antiguos de Europa, usado desde los tiempos del Sacro Imperio.</t>
         </is>
       </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Automóviles, maquinaria, química, productos farmacéuticos</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="80" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
@@ -1572,6 +1663,11 @@
           <t>Reúne los símbolos de los reinos históricos: Castilla (castillo), León (león), Aragón (franjas), Navarra (cadenas) y Granada (granada). Entre las columnas de Hércules.</t>
         </is>
       </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, aceite de oliva, vino, frutas y hortalizas</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="80" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
@@ -1629,6 +1725,11 @@
           <t>Francia no tiene un escudo oficial único actual, pero usa un emblema con un haz de lictor (unidad), ramas de roble (sabiduría) y olivo (paz), con las iniciales 'RF'.</t>
         </is>
       </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Aviones, vino, cosméticos, productos de lujo</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="80" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
@@ -1686,6 +1787,11 @@
           <t>Una estrella blanca de cinco puntas (Stella d'Italia) sobre una rueda dentada (el trabajo), rodeada por una rama de olivo (paz) y una de roble (fuerza).</t>
         </is>
       </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Maquinaria, vehículos, vino, moda y textiles</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="80" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
@@ -1743,6 +1849,11 @@
           <t>Una cruz blanca sobre fondo azul, rodeada por dos ramas de laurel. La cruz simboliza la fe ortodoxa y el laurel, el honor y la victoria.</t>
         </is>
       </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Aceite de oliva, petróleo refinado, pescado, aluminio</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="80" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
@@ -1800,6 +1911,11 @@
           <t>Cinco escudetes azules con puntos blancos (las 'quinas', cinco batallas cristianas) sobre siete castillos dorados (las plazas conquistadas a los moros), en la esfera armilar.</t>
         </is>
       </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, vino, corcho, calzado</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="80" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
@@ -1857,6 +1973,11 @@
           <t>Tres leones dorados (Inglaterra), un león rojo (Escocia) y un arpa (Irlanda), sobre una corona. Sostenido por un león y un unicornio. Lema: 'Dieu et mon droit'.</t>
         </is>
       </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, whisky, maquinaria, productos farmacéuticos</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="80" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
@@ -1914,6 +2035,11 @@
           <t>Un león dorado con espada y haz de flechas (las provincias unidas) sobre campo azul con bloques dorados. Lema: 'Je maintiendrai' ('Yo mantendré').</t>
         </is>
       </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo refinado, gas natural, flores, quesos</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1971,6 +2097,11 @@
           <t>La misma cruz blanca sobre escudo rojo. La cruz se asocia históricamente a los cantones fundadores y hoy es símbolo universal de la Cruz Roja.</t>
         </is>
       </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Relojes, química, oro, productos farmacéuticos</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="80" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -2028,6 +2159,11 @@
           <t>Tres coronas doradas sobre fondo azul ('Tre Kronor'). Es uno de los emblemas nacionales más antiguos de Europa, utilizado desde el siglo XIV.</t>
         </is>
       </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Maquinaria, mineral de hierro, madera, vehículos</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="80" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -2085,6 +2221,11 @@
           <t>Un león dorado coronado, sosteniendo el hacha de San Olaf, sobre fondo rojo. Es uno de los escudos más antiguos de Europa, datado del siglo XIII.</t>
         </is>
       </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, gas natural, pescado (salmón), aluminio</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="80" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -2142,6 +2283,11 @@
           <t>Un águila blanca coronada con el pico y las garras doradas, sobre fondo rojo. Según la leyenda, el fundador Lech vio un águila blanca al elegir dónde establecerse.</t>
         </is>
       </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, maquinaria, muebles, carbón</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="80" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
@@ -2199,6 +2345,11 @@
           <t>Puerta de Tiananmén bajo cinco estrellas doradas (el pueblo y el partido), rodeada por espigas de trigo y arroz y una rueda dentada (agricultura e industria).</t>
         </is>
       </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Electrónica, maquinaria, textiles, acero</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="80" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
@@ -2256,6 +2407,11 @@
           <t>Japón no tiene escudo oficial, pero usa el crisantemo imperial de 16 pétalos dorados como emblema de la Casa Imperial desde hace más de mil años.</t>
         </is>
       </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, electrónica, maquinaria, acero</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="80" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
@@ -2313,6 +2469,11 @@
           <t>Adaptado del Capitel de los Leones de Ashoka: cuatro leones de espaldas sobre una base con una rueda. Lema en sánscrito: 'Satyameva Jayate' ('Solo la verdad triunfa').</t>
         </is>
       </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Productos refinados de petróleo, diamantes, arroz, textiles</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="80" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
@@ -2370,6 +2531,11 @@
           <t>Una flor de hibisco (Rosa de Sharon, flor nacional) con cinco pétalos rodeando al taegeuk. En la cinta se lee 'Daehan Minguk' (República de Corea).</t>
         </is>
       </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Semiconductores, vehículos, barcos, electrónica</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="80" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
@@ -2427,6 +2593,11 @@
           <t>Turquía no tiene escudo oficial, pero usa un emblema con la media luna y la estrella sobre fondo rojo, acompañado del nombre 'Türkiye Cumhuriyeti'.</t>
         </is>
       </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Vehículos, textiles, oro, maquinaria</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="80" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
@@ -2484,6 +2655,11 @@
           <t>El Garuda, ave mítica montura del dios Vishnu, es el emblema real. Representa el poder del rey y se usa como sello oficial del gobierno.</t>
         </is>
       </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Electrónica, vehículos, caucho, arroz</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="80" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -2541,6 +2717,11 @@
           <t>La Menorá (candelabro de siete brazos del Templo de Jerusalén), rodeada por dos ramas de olivo (paz) y la palabra 'Israel' en hebreo abajo.</t>
         </is>
       </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Diamantes, tecnología, productos farmacéuticos, química</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="80" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
@@ -2598,6 +2779,11 @@
           <t>Una estrella dorada sobre fondo rojo rodeada por espigas de arroz y una rueda dentada, representando la unión de agricultura e industria bajo el socialismo.</t>
         </is>
       </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Electrónica, textiles, calzado, café</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="80" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -2655,6 +2841,11 @@
           <t>El Águila Dorada de Saladino, héroe medieval, sostiene un pergamino con el nombre del país en árabe. Representa fuerza, soberanía y la historia árabe.</t>
         </is>
       </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, gas natural, oro, textiles</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="80" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -2712,6 +2903,11 @@
           <t>Dos figuras humanas saludándose (unidad) sobre un escudo con plantas autóctonas. Encima, el ave secretario y una flor de protea. Lema: 'Unidad en la diversidad' en lengua khoisan.</t>
         </is>
       </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Oro, platino, carbón, mineral de hierro</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="80" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
@@ -2769,6 +2965,11 @@
           <t>Un sol naciente sobre las montañas del Atlas y la estrella verde, sostenido por dos leones. En la cinta, un versículo del Corán: 'Si ayudas a Dios, Él te ayudará'.</t>
         </is>
       </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Fosfato, automóviles, textiles, cítricos</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="80" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
@@ -2826,6 +3027,11 @@
           <t>Un águila negra (fuerza) sobre un escudo negro con una 'Y' plateada (los ríos Níger y Benue). Sostenido por dos caballos blancos (dignidad). Flores de 'costus spectabilis' alrededor.</t>
         </is>
       </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Petróleo, gas natural, cacao, sésamo</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="80" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
@@ -2883,6 +3089,11 @@
           <t>Un gallo blanco sosteniendo un hacha (lucha por la libertad), sobre un escudo masái con lanzas cruzadas. Lema en suajili: 'Harambee' ('Trabajemos juntos').</t>
         </is>
       </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Té, café, flores cortadas, horticultura</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="80" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
@@ -2938,6 +3149,11 @@
       <c r="K43" s="4" t="inlineStr">
         <is>
           <t>Un león dorado (fuerza y dinastías africanas) y un baobab (el árbol sagrado). La estrella verde aparece arriba. Lema: 'Un peuple, un but, une foi' ('Un pueblo, una meta, una fe').</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Oro, fosfatos, pescado, maní</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quitar emojis, agregar fronteras y clima al Excel y al detalle, achicar botones de navegación
</commit_message>
<xml_diff>
--- a/BD_banderas.xlsx
+++ b/BD_banderas.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -489,6 +489,9 @@
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,6 +555,21 @@
           <t>Materias primas exportadas</t>
         </is>
       </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Países limítrofes</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Clima (tipo)</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Clima (descripción)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="80" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -614,6 +632,21 @@
           <t>Soja, maíz, carne vacuna, trigo</t>
         </is>
       </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Bolivia, Brasil, Chile, Paraguay, Uruguay</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Subtropical al norte, templado en la pampa y frío patagónico en el sur.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="80" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -676,6 +709,21 @@
           <t>Gas natural, zinc, estaño, plata</t>
         </is>
       </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Argentina, Brasil, Chile, Paraguay, Perú</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Andino y tropical</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Frío seco en el altiplano, tropical cálido en los llanos y la Amazonia.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -738,6 +786,21 @@
           <t>Soja, mineral de hierro, petróleo, café</t>
         </is>
       </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Argentina, Bolivia, Colombia, Guyana, Guyana Francesa, Paraguay, Perú, Surinam, Uruguay, Venezuela</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Predominio tropical y ecuatorial húmedo; subtropical en el extremo sur.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -800,6 +863,21 @@
           <t>Petróleo, oro, madera, trigo</t>
         </is>
       </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Frío continental</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Inviernos largos y rigurosos; ártico en el norte, templado cerca de las costas.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -862,6 +940,21 @@
           <t>Cobre, litio, frutas, salmón</t>
         </is>
       </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Argentina, Bolivia, Perú</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Diverso</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Desértico en el norte, mediterráneo en el centro, templado lluvioso y polar al sur.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -924,6 +1017,21 @@
           <t>Petróleo, café, carbón, flores</t>
         </is>
       </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Brasil, Ecuador, Panamá, Perú, Venezuela</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo en las zonas bajas; templado y frío en la cordillera andina.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -986,6 +1094,21 @@
           <t>Dispositivos médicos, banano, piña, café</t>
         </is>
       </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Nicaragua, Panamá</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo todo el año con estación seca y estación lluviosa marcadas.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
@@ -1048,6 +1171,21 @@
           <t>Níquel, tabaco, azúcar, ron</t>
         </is>
       </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Sin fronteras terrestres (isla)</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo; temporada de huracanes entre junio y noviembre.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
@@ -1110,6 +1248,21 @@
           <t>Petróleo, banano, camarón, cacao</t>
         </is>
       </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Colombia, Perú</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Ecuatorial</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>Húmedo en la costa y la Amazonia; templado en la sierra andina.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
@@ -1172,6 +1325,21 @@
           <t>Petróleo, aviones, maíz, soja</t>
         </is>
       </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Canadá, México</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>De ártico en Alaska a tropical en Florida; continental, mediterráneo y desértico.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
@@ -1234,6 +1402,21 @@
           <t>Café, azúcar, banano, cardamomo</t>
         </is>
       </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Belice, El Salvador, Honduras, México</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>Cálido en las costas y templado de montaña en el altiplano central.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -1296,6 +1479,21 @@
           <t>Vehículos, petróleo, electrónica, aguacate</t>
         </is>
       </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Belice, Estados Unidos, Guatemala</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Desértico al norte, tropical al sur y templado en las mesetas centrales.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
@@ -1358,6 +1556,21 @@
           <t>Cobre, banano, azúcar, café</t>
         </is>
       </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Colombia, Costa Rica</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>Caluroso y húmedo durante todo el año, con estación lluviosa marcada.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
@@ -1420,6 +1633,21 @@
           <t>Cobre, oro, zinc, harina de pescado</t>
         </is>
       </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Bolivia, Brasil, Chile, Colombia, Ecuador</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Desértico en la costa, frío de montaña en los Andes y tropical en la selva.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="80" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
@@ -1482,6 +1710,21 @@
           <t>Soja, carne vacuna, maíz, energía eléctrica</t>
         </is>
       </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Argentina, Bolivia, Brasil</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Subtropical</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo al este; semiárido y caluroso en el Chaco occidental.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="80" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
@@ -1544,6 +1787,21 @@
           <t>Carne vacuna, soja, celulosa, lácteos</t>
         </is>
       </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Argentina, Brasil</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Templado</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Clima templado con cuatro estaciones suaves y humedad del Río de la Plata.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
@@ -1606,6 +1864,21 @@
           <t>Automóviles, maquinaria, química, productos farmacéuticos</t>
         </is>
       </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Austria, Bélgica, Chequia, Dinamarca, Francia, Luxemburgo, Países Bajos, Polonia, Suiza</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Templado</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>Oceánico suave en el norte y continental con inviernos fríos en el sur y este.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="80" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
@@ -1668,6 +1941,21 @@
           <t>Vehículos, aceite de oliva, vino, frutas y hortalizas</t>
         </is>
       </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Andorra, Francia, Portugal, Marruecos, Gibraltar</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Veranos cálidos y secos, inviernos suaves; oceánico en el norte y semiárido en el sureste.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="80" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
@@ -1730,6 +2018,21 @@
           <t>Aviones, vino, cosméticos, productos de lujo</t>
         </is>
       </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Alemania, Andorra, Bélgica, España, Italia, Luxemburgo, Mónaco, Suiza</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Templado</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>Oceánico en el oeste, continental en el interior y mediterráneo en el sur.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="80" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
@@ -1792,6 +2095,21 @@
           <t>Maquinaria, vehículos, vino, moda y textiles</t>
         </is>
       </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Austria, Eslovenia, Francia, San Marino, Suiza, Vaticano</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Veranos calurosos y secos; inviernos fríos en los Alpes y suaves al sur.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="80" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
@@ -1854,6 +2172,21 @@
           <t>Aceite de oliva, petróleo refinado, pescado, aluminio</t>
         </is>
       </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Albania, Bulgaria, Macedonia del Norte, Turquía</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>Veranos muy cálidos y secos; inviernos suaves y lluviosos en la costa.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="80" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
@@ -1916,6 +2249,21 @@
           <t>Vehículos, vino, corcho, calzado</t>
         </is>
       </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Suave y húmedo en el norte, caluroso y seco en el sur durante el verano.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="80" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
@@ -1978,6 +2326,21 @@
           <t>Petróleo, whisky, maquinaria, productos farmacéuticos</t>
         </is>
       </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Irlanda</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Oceánico</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>Lluvioso y templado todo el año, con veranos suaves e inviernos frescos.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="80" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
@@ -2040,6 +2403,21 @@
           <t>Petróleo refinado, gas natural, flores, quesos</t>
         </is>
       </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Alemania, Bélgica</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Oceánico</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Templado, húmedo y ventoso; veranos frescos e inviernos suaves.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -2102,6 +2480,21 @@
           <t>Relojes, química, oro, productos farmacéuticos</t>
         </is>
       </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>Alemania, Austria, Francia, Italia, Liechtenstein</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Alpino</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Templado en los valles, frío y nevado en las zonas de montaña durante el invierno.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="80" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -2164,6 +2557,21 @@
           <t>Maquinaria, mineral de hierro, madera, vehículos</t>
         </is>
       </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>Finlandia, Noruega</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Frío continental</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Inviernos largos y fríos, veranos cortos y suaves; subártico en el norte.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="80" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -2226,6 +2634,21 @@
           <t>Petróleo, gas natural, pescado (salmón), aluminio</t>
         </is>
       </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Finlandia, Rusia, Suecia</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Frío oceánico</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>Templado en la costa por la corriente del Golfo; subártico en el interior y norte.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="80" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -2288,6 +2711,21 @@
           <t>Vehículos, maquinaria, muebles, carbón</t>
         </is>
       </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Alemania, Bielorrusia, Chequia, Eslovaquia, Lituania, Rusia, Ucrania</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Continental templado</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Inviernos fríos y veranos cálidos, con influencia tanto marítima como continental.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="80" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
@@ -2350,6 +2788,21 @@
           <t>Electrónica, maquinaria, textiles, acero</t>
         </is>
       </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>Afganistán, Bután, Corea del Norte, India, Kazajistán, Kirguistán, Laos, Mongolia, Myanmar, Nepal, Pakistán, Rusia, Tayikistán, Vietnam</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>Continental seco en el norte y oeste; monzónico subtropical en el sur y este.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="80" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
@@ -2412,6 +2865,21 @@
           <t>Vehículos, electrónica, maquinaria, acero</t>
         </is>
       </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>Sin fronteras terrestres (isla)</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Templado monzónico</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>Cuatro estaciones marcadas; subtropical al sur y subártico al norte (Hokkaido).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="80" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
@@ -2474,6 +2942,21 @@
           <t>Productos refinados de petróleo, diamantes, arroz, textiles</t>
         </is>
       </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Bangladés, Bután, China, Myanmar, Nepal, Pakistán</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Monzónico</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Monzones de verano con lluvias intensas; tropical al sur y frío en el Himalaya.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="80" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
@@ -2536,6 +3019,21 @@
           <t>Semiconductores, vehículos, barcos, electrónica</t>
         </is>
       </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Corea del Norte</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Templado</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Cuatro estaciones bien definidas; veranos cálidos y húmedos, inviernos fríos.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="80" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
@@ -2598,6 +3096,21 @@
           <t>Vehículos, textiles, oro, maquinaria</t>
         </is>
       </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Armenia, Azerbaiyán, Bulgaria, Georgia, Grecia, Irak, Irán, Siria</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo en la costa, continental en el interior y más seco hacia el este.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="80" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
@@ -2660,6 +3173,21 @@
           <t>Electrónica, vehículos, caucho, arroz</t>
         </is>
       </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Camboya, Laos, Malasia, Myanmar</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo con monzones; estación lluviosa de mayo a octubre.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="80" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -2722,6 +3250,21 @@
           <t>Diamantes, tecnología, productos farmacéuticos, química</t>
         </is>
       </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>Egipto, Jordania, Líbano, Siria</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>Veranos calurosos y secos; inviernos suaves y lluviosos; desértico al sur (Néguev).</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="80" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
@@ -2784,6 +3327,21 @@
           <t>Electrónica, textiles, calzado, café</t>
         </is>
       </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Camboya, China, Laos</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Tropical monzónico</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo con monzones; más templado en las tierras altas del norte.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="80" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -2846,6 +3404,21 @@
           <t>Petróleo, gas natural, oro, textiles</t>
         </is>
       </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>Israel, Libia, Sudán</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Desértico</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>Muy seco y caluroso; valle del Nilo más templado y lluvias escasas en la costa.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="80" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -2908,6 +3481,21 @@
           <t>Oro, platino, carbón, mineral de hierro</t>
         </is>
       </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Botsuana, Esuatini, Lesoto, Mozambique, Namibia, Zimbabue</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo en el Cabo, semiárido en el interior y subtropical en la costa este.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="80" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
@@ -2970,6 +3558,21 @@
           <t>Fosfato, automóviles, textiles, cítricos</t>
         </is>
       </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>Argelia, España, Mauritania</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Mediterráneo y desértico</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>Suave en la costa; continental en el interior y desértico hacia el Sáhara.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="80" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
@@ -3032,6 +3635,21 @@
           <t>Petróleo, gas natural, cacao, sésamo</t>
         </is>
       </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>Benín, Camerún, Chad, Níger</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Ecuatorial húmedo en el sur y sabana más seca en el norte del país.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="80" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
@@ -3094,6 +3712,21 @@
           <t>Té, café, flores cortadas, horticultura</t>
         </is>
       </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>Etiopía, Somalia, Sudán del Sur, Tanzania, Uganda</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>Cálido todo el año; seco en el norte y más húmedo en las tierras altas centrales.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="80" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
@@ -3154,6 +3787,21 @@
       <c r="L43" s="4" t="inlineStr">
         <is>
           <t>Oro, fosfatos, pescado, maní</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Gambia, Guinea, Guinea-Bisáu, Malí, Mauritania</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>Tropical seco</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>Sabana con estación seca larga y estación lluviosa corta entre junio y octubre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Oceania (Australia, Nueva Zelanda, Papua Nueva Guinea, Fiji) + arreglar diseno barra puntaje en modal
</commit_message>
<xml_diff>
--- a/BD_banderas.xlsx
+++ b/BD_banderas.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +75,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3806,48 +3812,312 @@
       </c>
     </row>
     <row r="44" ht="80" customHeight="1">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>OC-01AU</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Oceanía</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>1 de enero</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>26.5M</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>50.7%</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>49.3%</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>Azul, Rojo, Blanco</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Azul, con la Union Jack británica en la esquina, recordando su historia colonial. La estrella grande de 7 puntas representa los 6 estados y los territorios. A la derecha, la constelación de la Cruz del Sur, visible desde el hemisferio sur.</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>Un canguro y un emú (animales que casi no pueden caminar hacia atrás, símbolo de progreso) sostienen un escudo con los símbolos de los 6 estados, sobre una rama de acacia dorada, flor nacional.</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Hierro, carbón, oro, gas natural, trigo, lana</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>(isla / archipiélago)</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>Desértico en el interior ('outback'), tropical en el norte y templado suave en las costas del sur y sureste.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="80" customHeight="1">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>OC-02NZ</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Nueva Zelanda</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Wellington</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Oceanía</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>6 de febrero</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>5.2M</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>50.6%</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>49.4%</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Azul, Rojo, Blanco</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Azul, con la Union Jack británica en la esquina. Las 4 estrellas rojas con borde blanco representan la Cruz del Sur, constelación visible en el cielo del hemisferio sur.</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Una mujer europea con la bandera y un jefe maorí con un bastón tradicional sostienen un escudo con 4 estrellas, un barco, una oveja, trigo, martillos y la Corona, símbolos de la historia y economía del país.</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Leche en polvo, mantequilla, carne de cordero, kiwi, vino</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>(isla / archipiélago)</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>Oceánico templado</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>Suave y lluvioso todo el año; veranos frescos e inviernos nevados en los Alpes del Sur.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="80" customHeight="1">
-      <c r="A46" s="1" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>OC-03PG</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Papúa Nueva Guinea</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Port Moresby</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Oceanía</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>16 de septiembre</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>10.1M</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>49.0%</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>51.0%</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>Rojo, Negro, Amarillo, Blanco</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Dividida en diagonal. La mitad roja con un Ave del Paraíso dorada, símbolo nacional famoso por sus plumas. La mitad negra con 5 estrellas blancas que forman la Cruz del Sur.</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Un Ave del Paraíso sobre una lanza tradicional y un tambor kundu, representando la cultura, las costumbres ancestrales y la fauna única del país.</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>Oro, cobre, gas natural, petróleo, café, aceite de palma</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>Tropical lluvioso</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y muy húmedo todo el año, con monzones; más fresco en las montañas del interior.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="80" customHeight="1">
-      <c r="A47" s="1" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>OC-04FJ</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Suva</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Oceanía</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>10 de octubre</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>0.9M</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>49.4%</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>50.6%</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Celeste, Azul, Rojo, Blanco, Amarillo</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Celeste como el océano Pacífico, con la Union Jack británica recordando el pasado colonial. A la derecha, una parte del escudo nacional con una paloma de la paz, caña de azúcar, coco y bananas.</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Una cruz roja con un león dorado arriba sosteniendo un coco, y cuatro secciones con caña de azúcar, un coco, una paloma de la paz y un racimo de bananas: productos y símbolos fundamentales de la isla.</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Caña de azúcar, agua embotellada, pescado, coco, oro</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>(isla / archipiélago)</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>Tropical oceánico</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>Cálido y húmedo todo el año, con lluvias abundantes y ciclones tropicales entre noviembre y abril.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="80" customHeight="1">
       <c r="A48" s="1" t="n"/>

</xml_diff>